<commit_message>
Added Literatures and update sample_data spread sheet
</commit_message>
<xml_diff>
--- a/results/StudyDetails.xlsx
+++ b/results/StudyDetails.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manjulat/Projects/Araichi/SkinDataAnalysis/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A490D22C-3CA4-3340-B9DA-69F40642EEA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E64460C-E1CA-734E-BE98-CB7473DA012C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1820" yWindow="660" windowWidth="15680" windowHeight="16680" activeTab="1" xr2:uid="{25722A3C-8689-2743-954C-0104D0233038}"/>
+    <workbookView xWindow="1820" yWindow="660" windowWidth="23540" windowHeight="16680" xr2:uid="{25722A3C-8689-2743-954C-0104D0233038}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="175">
   <si>
     <t>Study</t>
   </si>
@@ -313,9 +313,6 @@
     <t>atopic comorbidities: Allergic rhinoconjunctivitis, asthma</t>
   </si>
   <si>
-    <t>version 3 (10x Genomics)</t>
-  </si>
-  <si>
     <t>Medical University of Vienna</t>
   </si>
   <si>
@@ -553,9 +550,6 @@
     <t>1054 </t>
   </si>
   <si>
-    <t xml:space="preserve">10 AD </t>
-  </si>
-  <si>
     <t>Non-lesional</t>
   </si>
   <si>
@@ -566,6 +560,9 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>3' v3 (10x Genomics)</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +998,7 @@
         <v>21</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>2</v>
@@ -1051,7 +1048,7 @@
         <v>11</v>
       </c>
       <c r="J2" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K2" s="4" t="s">
         <v>67</v>
@@ -1083,10 +1080,10 @@
         <v>13</v>
       </c>
       <c r="J3" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1112,10 +1109,10 @@
         <v>15</v>
       </c>
       <c r="J4" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="K4" s="4" t="s">
         <v>91</v>
-      </c>
-      <c r="K4" s="4" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1142,39 +1139,42 @@
         <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B6">
         <v>10</v>
       </c>
-      <c r="C6" t="s">
-        <v>171</v>
+      <c r="D6">
+        <v>10</v>
       </c>
       <c r="F6" s="1">
         <v>19379</v>
       </c>
+      <c r="G6" s="1">
+        <v>22176</v>
+      </c>
       <c r="H6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
   </sheetData>
@@ -1199,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C1" t="s">
         <v>24</v>
@@ -1768,22 +1768,22 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B23" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E23" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="G23" s="8">
         <v>3663</v>
@@ -1794,22 +1794,22 @@
     </row>
     <row r="24" spans="1:8">
       <c r="A24" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B24" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E24" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="G24" s="8">
         <v>2859</v>
@@ -1820,22 +1820,22 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B25" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E25" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="F25" s="4" t="s">
-        <v>108</v>
       </c>
       <c r="G25" s="8">
         <v>4653</v>
@@ -1846,13 +1846,13 @@
     </row>
     <row r="26" spans="1:8">
       <c r="A26" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B26" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>19</v>
@@ -1861,7 +1861,7 @@
         <v>64</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G26" s="8">
         <v>3802</v>
@@ -1872,22 +1872,22 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B27" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E27" s="4" t="s">
         <v>64</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G27" s="8">
         <v>4084</v>
@@ -1898,22 +1898,22 @@
     </row>
     <row r="28" spans="1:8">
       <c r="A28" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B28" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E28" s="4" t="s">
         <v>64</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G28" s="8">
         <v>3719</v>
@@ -1924,22 +1924,22 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B29" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E29" s="4" t="s">
         <v>64</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G29" s="8">
         <v>2254</v>
@@ -1950,22 +1950,22 @@
     </row>
     <row r="30" spans="1:8">
       <c r="A30" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G30" s="8">
         <v>4846</v>
@@ -1976,19 +1976,19 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>89</v>
@@ -2002,19 +2002,19 @@
     </row>
     <row r="32" spans="1:8">
       <c r="A32" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>89</v>
@@ -2028,19 +2028,19 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F33" s="4" t="s">
         <v>89</v>
@@ -2054,22 +2054,22 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B34" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G34" s="8">
         <v>5628</v>
@@ -2080,22 +2080,22 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G35" s="8">
         <v>5104</v>
@@ -2106,22 +2106,22 @@
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G36" s="8">
         <v>6246</v>
@@ -2132,22 +2132,22 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G37" s="8">
         <v>5555</v>
@@ -2158,19 +2158,19 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F38" s="4" t="s">
         <v>89</v>
@@ -2184,19 +2184,19 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>89</v>
@@ -2210,19 +2210,19 @@
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B40" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F40" s="4" t="s">
         <v>89</v>
@@ -2236,19 +2236,19 @@
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B41" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F41" s="4" t="s">
         <v>89</v>
@@ -2262,19 +2262,19 @@
     </row>
     <row r="42" spans="1:9">
       <c r="A42" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>89</v>
@@ -2288,22 +2288,22 @@
     </row>
     <row r="43" spans="1:9">
       <c r="A43" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G43" s="8">
         <v>5455</v>
@@ -2314,22 +2314,22 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G44" s="8">
         <v>9737</v>
@@ -2340,48 +2340,48 @@
     </row>
     <row r="45" spans="1:9">
       <c r="A45" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>89</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F46" s="4" t="s">
         <v>89</v>
@@ -2390,24 +2390,24 @@
         <v>1499</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>89</v>
@@ -2416,24 +2416,24 @@
         <v>1570</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F48" s="4" t="s">
         <v>89</v>
@@ -2442,24 +2442,24 @@
         <v>4562</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F49" s="4" t="s">
         <v>89</v>
@@ -2468,24 +2468,24 @@
         <v>2976</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="50" spans="1:8">
       <c r="A50" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>89</v>
@@ -2494,24 +2494,24 @@
         <v>489</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F51" s="4" t="s">
         <v>89</v>
@@ -2520,24 +2520,24 @@
         <v>1866</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="52" spans="1:8">
       <c r="A52" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>89</v>
@@ -2546,24 +2546,24 @@
         <v>2478</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>89</v>
@@ -2572,24 +2572,24 @@
         <v>1942</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="54" spans="1:8">
       <c r="A54" s="4" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>89</v>
@@ -2598,7 +2598,7 @@
         <v>943</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>